<commit_message>
Add a .NET and Angular variant of the workshop; move the Python kit to demo/python-fastapi
WALKTHROUGH-dotnet.md, the ccw5gd deck, workbook and pre-work, the Northwind Dispatch practice kit
(ASP.NET Core 10 and Angular 19, six cases, history as a git bundle), and a cross-platform harness
(templates/run-case.cs) that runs every case in its own Docker container, on its own clone.

The Python kit moves from demo/ to demo/python-fastapi/; demo/README.md now lists both kits.
Eval runs in both kits now leave personal setup out (--setting-sources project,local,
--strict-mcp-config, --no-session-persistence, and hooks and auto memory off), and the tracker's
"How isolated" list gains "Container per run".
</commit_message>
<xml_diff>
--- a/templates/foundation-evaluation-tracker.xlsx
+++ b/templates/foundation-evaluation-tracker.xlsx
@@ -847,7 +847,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Fresh worktree: every baseline run uses a new git worktree from a clone that stops at the commit before the pull request, run with the eval-run settings file, so no run sees another's edits.  claude plugin eval: for later re-runs, once the foundation's skills ship in a plugin; the plugin's eval suite runs in a temporary home and workspace with only the plugin loaded.</t>
+          <t>Fresh worktree: every baseline run uses a new git worktree from a clone that stops at the commit before the pull request, run with the eval-run settings file, so no run sees another's edits.  Container per run: the .NET and Angular kit's run-case.cs gives every run its own clone of the case branch and its own Docker containers, which see that clone and nothing else.  claude plugin eval: for later re-runs, once the foundation's skills ship in a plugin; the plugin's eval suite runs in a temporary home and workspace with only the plugin loaded.</t>
         </is>
       </c>
     </row>
@@ -19386,7 +19386,7 @@
       <formula1>"Pass,Fail,Can't tell"</formula1>
     </dataValidation>
     <dataValidation sqref="H4:H1004" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Fresh worktree,claude plugin eval"</formula1>
+      <formula1>"Fresh worktree,Container per run,claude plugin eval"</formula1>
     </dataValidation>
     <dataValidation sqref="A5:A1004" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Eval Cases'!$A$5:$A$104</formula1>

</xml_diff>

<commit_message>
Apply the participant walkthrough review fixes to both kits
Per-task pass-rate exit criterion in the tracker and docs; run-case.cs
setupEnv/setupFiles for private feeds, model variables, and the credential
source printed in Claude Code's precedence order; walkthrough, workbook,
and pre-work fixes for both audiences; .gitattributes for line endings.
</commit_message>
<xml_diff>
--- a/templates/foundation-evaluation-tracker.xlsx
+++ b/templates/foundation-evaluation-tracker.xlsx
@@ -20966,7 +20966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S103"/>
+  <dimension ref="A1:T103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20984,6 +20984,7 @@
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="8" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21072,6 +21073,11 @@
           <t>Pass rate</t>
         </is>
       </c>
+      <c r="T3" s="10" t="inlineStr">
+        <is>
+          <t>Meets the target?</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="21">
@@ -21135,6 +21141,10 @@
         <f>IF(O4="","",IF(Q4=0,"",R4/Q4))</f>
         <v/>
       </c>
+      <c r="T4" s="21">
+        <f>IF(OR(S4="",'Exit Criteria'!$C$5=""),"",IF(S4&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="21">
@@ -21198,6 +21208,10 @@
         <f>IF(O5="","",IF(Q5=0,"",R5/Q5))</f>
         <v/>
       </c>
+      <c r="T5" s="21">
+        <f>IF(OR(S5="",'Exit Criteria'!$C$5=""),"",IF(S5&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="21">
@@ -21261,6 +21275,10 @@
         <f>IF(O6="","",IF(Q6=0,"",R6/Q6))</f>
         <v/>
       </c>
+      <c r="T6" s="21">
+        <f>IF(OR(S6="",'Exit Criteria'!$C$5=""),"",IF(S6&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="21">
@@ -21324,6 +21342,10 @@
         <f>IF(O7="","",IF(Q7=0,"",R7/Q7))</f>
         <v/>
       </c>
+      <c r="T7" s="21">
+        <f>IF(OR(S7="",'Exit Criteria'!$C$5=""),"",IF(S7&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="21">
@@ -21387,6 +21409,10 @@
         <f>IF(O8="","",IF(Q8=0,"",R8/Q8))</f>
         <v/>
       </c>
+      <c r="T8" s="21">
+        <f>IF(OR(S8="",'Exit Criteria'!$C$5=""),"",IF(S8&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="21">
@@ -21450,6 +21476,10 @@
         <f>IF(O9="","",IF(Q9=0,"",R9/Q9))</f>
         <v/>
       </c>
+      <c r="T9" s="21">
+        <f>IF(OR(S9="",'Exit Criteria'!$C$5=""),"",IF(S9&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="21">
@@ -21513,6 +21543,10 @@
         <f>IF(O10="","",IF(Q10=0,"",R10/Q10))</f>
         <v/>
       </c>
+      <c r="T10" s="21">
+        <f>IF(OR(S10="",'Exit Criteria'!$C$5=""),"",IF(S10&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="21">
@@ -21576,6 +21610,10 @@
         <f>IF(O11="","",IF(Q11=0,"",R11/Q11))</f>
         <v/>
       </c>
+      <c r="T11" s="21">
+        <f>IF(OR(S11="",'Exit Criteria'!$C$5=""),"",IF(S11&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="21">
@@ -21639,6 +21677,10 @@
         <f>IF(O12="","",IF(Q12=0,"",R12/Q12))</f>
         <v/>
       </c>
+      <c r="T12" s="21">
+        <f>IF(OR(S12="",'Exit Criteria'!$C$5=""),"",IF(S12&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="21">
@@ -21702,6 +21744,10 @@
         <f>IF(O13="","",IF(Q13=0,"",R13/Q13))</f>
         <v/>
       </c>
+      <c r="T13" s="21">
+        <f>IF(OR(S13="",'Exit Criteria'!$C$5=""),"",IF(S13&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="21">
@@ -21765,6 +21811,10 @@
         <f>IF(O14="","",IF(Q14=0,"",R14/Q14))</f>
         <v/>
       </c>
+      <c r="T14" s="21">
+        <f>IF(OR(S14="",'Exit Criteria'!$C$5=""),"",IF(S14&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="21">
@@ -21828,6 +21878,10 @@
         <f>IF(O15="","",IF(Q15=0,"",R15/Q15))</f>
         <v/>
       </c>
+      <c r="T15" s="21">
+        <f>IF(OR(S15="",'Exit Criteria'!$C$5=""),"",IF(S15&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="21">
@@ -21882,6 +21936,10 @@
         <f>IF(O16="","",IF(Q16=0,"",R16/Q16))</f>
         <v/>
       </c>
+      <c r="T16" s="21">
+        <f>IF(OR(S16="",'Exit Criteria'!$C$5=""),"",IF(S16&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="21">
@@ -21936,6 +21994,10 @@
         <f>IF(O17="","",IF(Q17=0,"",R17/Q17))</f>
         <v/>
       </c>
+      <c r="T17" s="21">
+        <f>IF(OR(S17="",'Exit Criteria'!$C$5=""),"",IF(S17&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="21">
@@ -21990,6 +22052,10 @@
         <f>IF(O18="","",IF(Q18=0,"",R18/Q18))</f>
         <v/>
       </c>
+      <c r="T18" s="21">
+        <f>IF(OR(S18="",'Exit Criteria'!$C$5=""),"",IF(S18&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="21">
@@ -22044,6 +22110,10 @@
         <f>IF(O19="","",IF(Q19=0,"",R19/Q19))</f>
         <v/>
       </c>
+      <c r="T19" s="21">
+        <f>IF(OR(S19="",'Exit Criteria'!$C$5=""),"",IF(S19&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="21">
@@ -22098,6 +22168,10 @@
         <f>IF(O20="","",IF(Q20=0,"",R20/Q20))</f>
         <v/>
       </c>
+      <c r="T20" s="21">
+        <f>IF(OR(S20="",'Exit Criteria'!$C$5=""),"",IF(S20&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="21">
@@ -22152,6 +22226,10 @@
         <f>IF(O21="","",IF(Q21=0,"",R21/Q21))</f>
         <v/>
       </c>
+      <c r="T21" s="21">
+        <f>IF(OR(S21="",'Exit Criteria'!$C$5=""),"",IF(S21&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="21">
@@ -22206,6 +22284,10 @@
         <f>IF(O22="","",IF(Q22=0,"",R22/Q22))</f>
         <v/>
       </c>
+      <c r="T22" s="21">
+        <f>IF(OR(S22="",'Exit Criteria'!$C$5=""),"",IF(S22&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="21">
@@ -22258,6 +22340,10 @@
       </c>
       <c r="S23" s="22">
         <f>IF(O23="","",IF(Q23=0,"",R23/Q23))</f>
+        <v/>
+      </c>
+      <c r="T23" s="21">
+        <f>IF(OR(S23="",'Exit Criteria'!$C$5=""),"",IF(S23&gt;='Exit Criteria'!$C$5,"Yes","No"))</f>
         <v/>
       </c>
     </row>
@@ -24988,6 +25074,14 @@
       <formula>"Yes"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T4:T23">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="0">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -26041,7 +26135,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Set before results come in. Rows 5 and 6 calculate from the Summary, and row 9 from Target Tasks. Set each target from the foundation's own week-1 baseline; Anthropic benchmarks are for comparison only. Row 4 is an example.</t>
+          <t>Set before results come in. Rows 5 and 6 calculate from the Summary, and row 9 from Target Tasks. Row 5 is judged per target task: each task's pass rate against the target, as the Summary's 'Meets the target?' column shows. Set each target from the foundation's own week-1 baseline; Anthropic benchmarks are for comparison only. Row 4 is an example.</t>
         </is>
       </c>
     </row>
@@ -26104,7 +26198,7 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Target-task pass rate</t>
+          <t>Target-task pass rate, per task (each target task must reach it)</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -26113,12 +26207,12 @@
         </is>
       </c>
       <c r="C5" s="26" t="n"/>
-      <c r="D5" s="27">
-        <f>Summary!M9</f>
+      <c r="D5" s="13">
+        <f>IF(OR(C5="",COUNT(Summary!$S$4:$S$23)=0),"",COUNTIF(Summary!$S$4:$S$23,"&gt;="&amp;C5)&amp;" of "&amp;COUNT(Summary!$S$4:$S$23)&amp;" target tasks at or above target")</f>
         <v/>
       </c>
       <c r="E5" s="13">
-        <f>IF(OR(C5="",D5=""),"Not yet measured",IF(D5&gt;=C5,"Yes","No"))</f>
+        <f>IF(OR(C5="",D5=""),"Not yet measured",IF(COUNTIF(Summary!$S$4:$S$23,"&gt;="&amp;C5)=COUNT(Summary!$S$4:$S$23),"Yes","No"))</f>
         <v/>
       </c>
       <c r="F5" s="12" t="n"/>

</xml_diff>